<commit_message>
docs: asset production guide and source art
Chat prompt workflow for generating gear images, the white-label homage
rule, updated gear references (Noise Gate, Orange Squeeze) and the
original Noise Gate source images.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/assets-equipamentos.xlsx
+++ b/docs/assets-equipamentos.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Boss NS-2 / ISP Decimator</t>
+          <t>Boss NS-2 (o Decay dele = nosso Release; sem o knob Mode)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>MXR Dyna Comp (compressor laranja)</t>
+          <t>MXR Dyna Comp (a versão laranja dos anos 70/80)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Inferido</t>
+          <t>Confirmado no código</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Threshold, Ratio, Attack, Release</t>
+          <t>Sensitivity, Output</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">

</xml_diff>